<commit_message>
Add orphan buy scanning and token balance retrieval to delayed_orders_strategy; update version to 1.3.0
</commit_message>
<xml_diff>
--- a/hype_stat.xlsx
+++ b/hype_stat.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,6 +622,114 @@
       </c>
       <c r="J5" t="n">
         <v>500.0133195084156</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:39:35</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>85495.5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Set TP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.00028</v>
+      </c>
+      <c r="E6" t="n">
+        <v>85778</v>
+      </c>
+      <c r="F6" t="n">
+        <v>451.02586</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0005696012000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>48.03036</v>
+      </c>
+      <c r="I6" t="n">
+        <v>499.7241993946</v>
+      </c>
+      <c r="J6" t="n">
+        <v>499.3008293635267</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:48:26</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>85682.5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pyramiding</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.00026</v>
+      </c>
+      <c r="E7" t="n">
+        <v>85628</v>
+      </c>
+      <c r="F7" t="n">
+        <v>451.02586</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0008294193</v>
+      </c>
+      <c r="H7" t="n">
+        <v>48.03036</v>
+      </c>
+      <c r="I7" t="n">
+        <v>522.0473758204</v>
+      </c>
+      <c r="J7" t="n">
+        <v>500.3929249134794</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:48:39</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>85678.5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Set TP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="E8" t="n">
+        <v>85828</v>
+      </c>
+      <c r="F8" t="n">
+        <v>428.76258</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0008294193</v>
+      </c>
+      <c r="H8" t="n">
+        <v>69.48736</v>
+      </c>
+      <c r="I8" t="n">
+        <v>499.82598149505</v>
+      </c>
+      <c r="J8" t="n">
+        <v>500.3695645808601</v>
       </c>
     </row>
   </sheetData>

</xml_diff>